<commit_message>
Fix Circulator Upload failures. Update Certificate upload template to 1.5
</commit_message>
<xml_diff>
--- a/routes/er-circulator-listings.xlsx
+++ b/routes/er-circulator-listings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\hi-er\routes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\orig\hi-er\routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C99476-8277-42A5-ADE7-73783AADD710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{630094C1-DB5A-46CE-96E1-A14D922F2F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6036" yWindow="1284" windowWidth="23040" windowHeight="14460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30030" yWindow="2130" windowWidth="25275" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
@@ -418,9 +418,6 @@
     <t>Do not enter any data here, only applicable on export</t>
   </si>
   <si>
-    <t>No Speed Control</t>
-  </si>
-  <si>
     <t>CP1: Wet Rotor</t>
   </si>
   <si>
@@ -443,9 +440,6 @@
   </si>
   <si>
     <t>External Input Signal and Other Controls</t>
-  </si>
-  <si>
-    <t>Manual Speed Controls</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -580,6 +574,12 @@
   </si>
   <si>
     <t>Yes/No</t>
+  </si>
+  <si>
+    <t>Full Speed</t>
+  </si>
+  <si>
+    <t>Manual Speed Control</t>
   </si>
 </sst>
 </file>
@@ -1197,9 +1197,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1261,32 +1258,35 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1703,43 +1703,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AL4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
-    <col min="6" max="6" width="28.6640625" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="13.33203125" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="28.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" customWidth="1"/>
     <col min="14" max="16" width="30" customWidth="1"/>
-    <col min="17" max="17" width="28.109375" customWidth="1"/>
+    <col min="17" max="17" width="28.140625" customWidth="1"/>
     <col min="18" max="18" width="14" customWidth="1"/>
-    <col min="19" max="19" width="13.6640625" customWidth="1"/>
-    <col min="20" max="20" width="14.44140625" customWidth="1"/>
-    <col min="21" max="21" width="14.33203125" customWidth="1"/>
-    <col min="22" max="22" width="15.6640625" customWidth="1"/>
-    <col min="23" max="23" width="17.33203125" customWidth="1"/>
-    <col min="24" max="25" width="14.33203125" customWidth="1"/>
-    <col min="26" max="26" width="17.33203125" customWidth="1"/>
-    <col min="27" max="29" width="19.109375" customWidth="1"/>
-    <col min="30" max="30" width="12.109375" customWidth="1"/>
-    <col min="31" max="31" width="14.109375" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="14.28515625" customWidth="1"/>
+    <col min="22" max="22" width="15.7109375" customWidth="1"/>
+    <col min="23" max="23" width="17.28515625" customWidth="1"/>
+    <col min="24" max="25" width="14.28515625" customWidth="1"/>
+    <col min="26" max="26" width="17.28515625" customWidth="1"/>
+    <col min="27" max="29" width="19.140625" customWidth="1"/>
+    <col min="30" max="30" width="12.140625" customWidth="1"/>
+    <col min="31" max="31" width="14.140625" customWidth="1"/>
     <col min="32" max="32" width="14" customWidth="1"/>
-    <col min="33" max="34" width="14.6640625" customWidth="1"/>
-    <col min="35" max="35" width="20.33203125" customWidth="1"/>
-    <col min="36" max="36" width="18.33203125" customWidth="1"/>
-    <col min="37" max="38" width="17.88671875" customWidth="1"/>
-    <col min="39" max="1025" width="8.44140625" customWidth="1"/>
+    <col min="33" max="34" width="14.7109375" customWidth="1"/>
+    <col min="35" max="35" width="20.28515625" customWidth="1"/>
+    <col min="36" max="36" width="18.28515625" customWidth="1"/>
+    <col min="37" max="38" width="17.85546875" customWidth="1"/>
+    <col min="39" max="1025" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="1" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:38" s="1" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="56" t="s">
         <v>0</v>
       </c>
@@ -1762,23 +1762,23 @@
       <c r="P1" s="57"/>
       <c r="Q1" s="57"/>
       <c r="R1" s="59" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="S1" s="59"/>
       <c r="T1" s="59"/>
       <c r="U1" s="59"/>
       <c r="V1" s="59" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="W1" s="59"/>
       <c r="X1" s="60" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Y1" s="60"/>
       <c r="Z1" s="60"/>
       <c r="AA1" s="60"/>
       <c r="AB1" s="61" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="AC1" s="61"/>
       <c r="AD1" s="62" t="s">
@@ -1791,19 +1791,19 @@
         <v>3</v>
       </c>
       <c r="AI1" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AJ1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AK1" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="AJ1" s="4" t="s">
+      <c r="AL1" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="AK1" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="AL1" s="6" t="s">
-        <v>94</v>
-      </c>
     </row>
-    <row r="2" spans="1:38" ht="35.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:38" ht="33" x14ac:dyDescent="0.25">
       <c r="A2" s="56"/>
       <c r="B2" s="56"/>
       <c r="C2" s="56"/>
@@ -1873,10 +1873,10 @@
         <v>14</v>
       </c>
       <c r="AI2" s="19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AJ2" s="19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AK2" s="20" t="s">
         <v>15</v>
@@ -1885,7 +1885,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="133.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:38" ht="133.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>16</v>
       </c>
@@ -1904,152 +1904,152 @@
       <c r="F3" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="N3" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="O3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="P3" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q3" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="R3" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="S3" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="T3" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="U3" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="V3" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="W3" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="X3" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="Y3" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="Z3" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA3" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="AB3" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="AC3" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD3" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE3" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF3" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG3" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH3" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI3" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="AJ3" s="41" t="s">
+        <v>82</v>
+      </c>
+      <c r="AK3" s="42" t="s">
+        <v>83</v>
+      </c>
+      <c r="AL3" s="42" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" ht="245.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="43"/>
+      <c r="B4" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="I3" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="O3" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="P3" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q3" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="R3" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="S3" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="T3" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="U3" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="V3" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="W3" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="X3" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA3" s="35" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB3" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="AC3" s="36" t="s">
-        <v>82</v>
-      </c>
-      <c r="AD3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE3" s="38" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF3" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG3" s="39" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH3" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI3" s="41" t="s">
-        <v>83</v>
-      </c>
-      <c r="AJ3" s="42" t="s">
-        <v>84</v>
-      </c>
-      <c r="AK3" s="43" t="s">
+      <c r="C4" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="45" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="N4" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="AL3" s="43" t="s">
+      <c r="O4" s="46" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="4" spans="1:38" ht="245.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="45" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" s="45" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="47" t="s">
-        <v>58</v>
-      </c>
-      <c r="I4" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="L4" s="48" t="s">
-        <v>39</v>
-      </c>
-      <c r="M4" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="N4" s="48" t="s">
+      <c r="P4" s="47" t="s">
         <v>87</v>
       </c>
-      <c r="O4" s="48" t="s">
+      <c r="Q4" s="48" t="s">
         <v>88</v>
-      </c>
-      <c r="P4" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q4" s="50" t="s">
-        <v>90</v>
       </c>
       <c r="R4" s="63" t="s">
         <v>41</v>
@@ -2077,19 +2077,19 @@
       <c r="AE4" s="58"/>
       <c r="AF4" s="58"/>
       <c r="AG4" s="58"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AH4" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="AI4" s="52" t="s">
+      <c r="AI4" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="AJ4" s="52" t="s">
+      <c r="AJ4" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="AK4" s="53" t="s">
+      <c r="AK4" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="AL4" s="53" t="s">
+      <c r="AL4" s="51" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
     <mergeCell ref="AB4:AC4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
@@ -2140,64 +2140,64 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.33203125" customWidth="1"/>
-    <col min="2" max="2" width="24.88671875" customWidth="1"/>
-    <col min="3" max="1025" width="8.44140625" customWidth="1"/>
+    <col min="1" max="1" width="40.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="3" max="1025" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="55" t="s">
+      <c r="C1" s="53" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2209,26 +2209,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{712FBA03-4FCA-480E-9824-0D062368D4BA}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B1">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B2" s="54">
-        <v>45768</v>
+        <v>94</v>
+      </c>
+      <c r="B2" s="52">
+        <v>46175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Circulator Upload failures. Update Certificate upload template to 1.5 (#26)
</commit_message>
<xml_diff>
--- a/routes/er-circulator-listings.xlsx
+++ b/routes/er-circulator-listings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\hi-er\routes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\orig\hi-er\routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C99476-8277-42A5-ADE7-73783AADD710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{630094C1-DB5A-46CE-96E1-A14D922F2F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6036" yWindow="1284" windowWidth="23040" windowHeight="14460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30030" yWindow="2130" windowWidth="25275" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
@@ -418,9 +418,6 @@
     <t>Do not enter any data here, only applicable on export</t>
   </si>
   <si>
-    <t>No Speed Control</t>
-  </si>
-  <si>
     <t>CP1: Wet Rotor</t>
   </si>
   <si>
@@ -443,9 +440,6 @@
   </si>
   <si>
     <t>External Input Signal and Other Controls</t>
-  </si>
-  <si>
-    <t>Manual Speed Controls</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -580,6 +574,12 @@
   </si>
   <si>
     <t>Yes/No</t>
+  </si>
+  <si>
+    <t>Full Speed</t>
+  </si>
+  <si>
+    <t>Manual Speed Control</t>
   </si>
 </sst>
 </file>
@@ -1197,9 +1197,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1261,32 +1258,35 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1703,43 +1703,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AL4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
-    <col min="6" max="6" width="28.6640625" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="13.33203125" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="28.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" customWidth="1"/>
     <col min="14" max="16" width="30" customWidth="1"/>
-    <col min="17" max="17" width="28.109375" customWidth="1"/>
+    <col min="17" max="17" width="28.140625" customWidth="1"/>
     <col min="18" max="18" width="14" customWidth="1"/>
-    <col min="19" max="19" width="13.6640625" customWidth="1"/>
-    <col min="20" max="20" width="14.44140625" customWidth="1"/>
-    <col min="21" max="21" width="14.33203125" customWidth="1"/>
-    <col min="22" max="22" width="15.6640625" customWidth="1"/>
-    <col min="23" max="23" width="17.33203125" customWidth="1"/>
-    <col min="24" max="25" width="14.33203125" customWidth="1"/>
-    <col min="26" max="26" width="17.33203125" customWidth="1"/>
-    <col min="27" max="29" width="19.109375" customWidth="1"/>
-    <col min="30" max="30" width="12.109375" customWidth="1"/>
-    <col min="31" max="31" width="14.109375" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="14.28515625" customWidth="1"/>
+    <col min="22" max="22" width="15.7109375" customWidth="1"/>
+    <col min="23" max="23" width="17.28515625" customWidth="1"/>
+    <col min="24" max="25" width="14.28515625" customWidth="1"/>
+    <col min="26" max="26" width="17.28515625" customWidth="1"/>
+    <col min="27" max="29" width="19.140625" customWidth="1"/>
+    <col min="30" max="30" width="12.140625" customWidth="1"/>
+    <col min="31" max="31" width="14.140625" customWidth="1"/>
     <col min="32" max="32" width="14" customWidth="1"/>
-    <col min="33" max="34" width="14.6640625" customWidth="1"/>
-    <col min="35" max="35" width="20.33203125" customWidth="1"/>
-    <col min="36" max="36" width="18.33203125" customWidth="1"/>
-    <col min="37" max="38" width="17.88671875" customWidth="1"/>
-    <col min="39" max="1025" width="8.44140625" customWidth="1"/>
+    <col min="33" max="34" width="14.7109375" customWidth="1"/>
+    <col min="35" max="35" width="20.28515625" customWidth="1"/>
+    <col min="36" max="36" width="18.28515625" customWidth="1"/>
+    <col min="37" max="38" width="17.85546875" customWidth="1"/>
+    <col min="39" max="1025" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="1" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:38" s="1" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="56" t="s">
         <v>0</v>
       </c>
@@ -1762,23 +1762,23 @@
       <c r="P1" s="57"/>
       <c r="Q1" s="57"/>
       <c r="R1" s="59" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="S1" s="59"/>
       <c r="T1" s="59"/>
       <c r="U1" s="59"/>
       <c r="V1" s="59" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="W1" s="59"/>
       <c r="X1" s="60" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Y1" s="60"/>
       <c r="Z1" s="60"/>
       <c r="AA1" s="60"/>
       <c r="AB1" s="61" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="AC1" s="61"/>
       <c r="AD1" s="62" t="s">
@@ -1791,19 +1791,19 @@
         <v>3</v>
       </c>
       <c r="AI1" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AJ1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AK1" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="AJ1" s="4" t="s">
+      <c r="AL1" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="AK1" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="AL1" s="6" t="s">
-        <v>94</v>
-      </c>
     </row>
-    <row r="2" spans="1:38" ht="35.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:38" ht="33" x14ac:dyDescent="0.25">
       <c r="A2" s="56"/>
       <c r="B2" s="56"/>
       <c r="C2" s="56"/>
@@ -1873,10 +1873,10 @@
         <v>14</v>
       </c>
       <c r="AI2" s="19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AJ2" s="19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AK2" s="20" t="s">
         <v>15</v>
@@ -1885,7 +1885,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="133.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:38" ht="133.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>16</v>
       </c>
@@ -1904,152 +1904,152 @@
       <c r="F3" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="N3" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="O3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="P3" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q3" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="R3" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="S3" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="T3" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="U3" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="V3" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="W3" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="X3" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="Y3" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="Z3" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA3" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="AB3" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="AC3" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD3" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE3" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF3" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG3" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH3" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI3" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="AJ3" s="41" t="s">
+        <v>82</v>
+      </c>
+      <c r="AK3" s="42" t="s">
+        <v>83</v>
+      </c>
+      <c r="AL3" s="42" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" ht="245.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="43"/>
+      <c r="B4" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="I3" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="O3" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="P3" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q3" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="R3" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="S3" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="T3" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="U3" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="V3" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="W3" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="X3" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA3" s="35" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB3" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="AC3" s="36" t="s">
-        <v>82</v>
-      </c>
-      <c r="AD3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE3" s="38" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF3" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG3" s="39" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH3" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI3" s="41" t="s">
-        <v>83</v>
-      </c>
-      <c r="AJ3" s="42" t="s">
-        <v>84</v>
-      </c>
-      <c r="AK3" s="43" t="s">
+      <c r="C4" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="45" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="N4" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="AL3" s="43" t="s">
+      <c r="O4" s="46" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="4" spans="1:38" ht="245.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="45" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" s="45" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="47" t="s">
-        <v>58</v>
-      </c>
-      <c r="I4" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="L4" s="48" t="s">
-        <v>39</v>
-      </c>
-      <c r="M4" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="N4" s="48" t="s">
+      <c r="P4" s="47" t="s">
         <v>87</v>
       </c>
-      <c r="O4" s="48" t="s">
+      <c r="Q4" s="48" t="s">
         <v>88</v>
-      </c>
-      <c r="P4" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q4" s="50" t="s">
-        <v>90</v>
       </c>
       <c r="R4" s="63" t="s">
         <v>41</v>
@@ -2077,19 +2077,19 @@
       <c r="AE4" s="58"/>
       <c r="AF4" s="58"/>
       <c r="AG4" s="58"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AH4" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="AI4" s="52" t="s">
+      <c r="AI4" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="AJ4" s="52" t="s">
+      <c r="AJ4" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="AK4" s="53" t="s">
+      <c r="AK4" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="AL4" s="53" t="s">
+      <c r="AL4" s="51" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
     <mergeCell ref="AB4:AC4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
@@ -2140,64 +2140,64 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.33203125" customWidth="1"/>
-    <col min="2" max="2" width="24.88671875" customWidth="1"/>
-    <col min="3" max="1025" width="8.44140625" customWidth="1"/>
+    <col min="1" max="1" width="40.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="3" max="1025" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="55" t="s">
+      <c r="C1" s="53" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2209,26 +2209,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{712FBA03-4FCA-480E-9824-0D062368D4BA}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B1">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B2" s="54">
-        <v>45768</v>
+        <v>94</v>
+      </c>
+      <c r="B2" s="52">
+        <v>46175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>